<commit_message>
chore: sync Nova upm-release-2026.08.20-01
</commit_message>
<xml_diff>
--- a/Assets/Samples/MainDemo/Excels/UIs/UIs.xlsx
+++ b/Assets/Samples/MainDemo/Excels/UIs/UIs.xlsx
@@ -2024,7 +2024,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>HybridCLR 3.2 业务 dll</t>
+          <t>HybridCLR 3.2 启动时业务 DLL</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -2075,17 +2075,17 @@
     <row r="35" ht="22" customHeight="1" s="6">
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>DemoIntegrationUiLocalizationView</t>
+          <t>DemoHybridClrRuntimeUpdateView</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Integration 4.1 UI+Localization</t>
+          <t>HybridCLR 3.4 运行时增量热更新</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>DemoIntegrationUiLocalizationView</t>
+          <t>DemoHybridClrRuntimeUpdateView</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -2103,17 +2103,17 @@
     <row r="36" ht="22" customHeight="1" s="6">
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>DemoIntegrationUiAssetView</t>
+          <t>DemoIntegrationUiLocalizationView</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Integration 4.2 UI+Asset</t>
+          <t>Integration 4.1 UI+Localization</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>DemoIntegrationUiAssetView</t>
+          <t>DemoIntegrationUiLocalizationView</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -2131,17 +2131,17 @@
     <row r="37" ht="22" customHeight="1" s="6">
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>DemoIntegrationProcedureAssetView</t>
+          <t>DemoIntegrationUiAssetView</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Integration 4.3 Procedure+Asset</t>
+          <t>Integration 4.2 UI+Asset</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>DemoIntegrationProcedureAssetView</t>
+          <t>DemoIntegrationUiAssetView</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Integration 4.4 Event+Network</t>
+          <t>Integration 4.3 Event+Network</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Integration 4.5 Config+HybridCLR</t>
+          <t>Integration 4.4 Config+HybridCLR</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">

</xml_diff>